<commit_message>
E-Com FC: add revenue recognition from other RN to E-com (+100 Nov, +100 Dec); total 6 345
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142u1JgEJ5Z4iqbgjpLWfcB
</commit_message>
<xml_diff>
--- a/E-Com_FC_Sep_fact_Oct-Dec_FC.xlsx
+++ b/E-Com_FC_Sep_fact_Oct-Dec_FC.xlsx
@@ -505,11 +505,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O6"/>
+  <dimension ref="B1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.5"/>
   <cols>
     <col width="8.7265625" customWidth="1" style="4" min="1" max="1"/>
-    <col width="29.1796875" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="44" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
     <col width="10.90625" customWidth="1" style="4" min="3" max="15"/>
     <col width="8.7265625" customWidth="1" style="4" min="16" max="16384"/>
   </cols>
@@ -755,65 +755,111 @@
       </c>
     </row>
     <row r="6" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Признание выручки с не наших РН на РН E-com</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="O6" s="9">
+        <f>SUM(C6:N6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="13.5" customHeight="1" thickTop="1">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Итог</t>
         </is>
       </c>
-      <c r="C6" s="11">
-        <f>SUM(C4:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="11">
-        <f>SUM(D4:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="11">
-        <f>SUM(E4:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="11">
-        <f>SUM(F4:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="11">
-        <f>SUM(G4:G5)</f>
-        <v/>
-      </c>
-      <c r="H6" s="11">
-        <f>SUM(H4:H5)</f>
-        <v/>
-      </c>
-      <c r="I6" s="11">
-        <f>SUM(I4:I5)</f>
-        <v/>
-      </c>
-      <c r="J6" s="11">
-        <f>SUM(J4:J5)</f>
-        <v/>
-      </c>
-      <c r="K6" s="11">
-        <f>SUM(K4:K5)</f>
-        <v/>
-      </c>
-      <c r="L6" s="11">
-        <f>SUM(L4:L5)</f>
-        <v/>
-      </c>
-      <c r="M6" s="11">
-        <f>SUM(M4:M5)</f>
-        <v/>
-      </c>
-      <c r="N6" s="11">
-        <f>SUM(N4:N5)</f>
-        <v/>
-      </c>
-      <c r="O6" s="11">
-        <f>SUM(O4:O5)</f>
+      <c r="C7" s="11">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>SUM(E4:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>SUM(F4:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>SUM(G4:G6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
+        <f>SUM(H4:H6)</f>
+        <v/>
+      </c>
+      <c r="I7" s="11">
+        <f>SUM(I4:I6)</f>
+        <v/>
+      </c>
+      <c r="J7" s="11">
+        <f>SUM(J4:J6)</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
+        <f>SUM(K4:K6)</f>
+        <v/>
+      </c>
+      <c r="L7" s="11">
+        <f>SUM(L4:L6)</f>
+        <v/>
+      </c>
+      <c r="M7" s="11">
+        <f>SUM(M4:M6)</f>
+        <v/>
+      </c>
+      <c r="N7" s="11">
+        <f>SUM(N4:N6)</f>
+        <v/>
+      </c>
+      <c r="O7" s="11">
+        <f>SUM(O4:O6)</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="13" customHeight="1" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>